<commit_message>
Split out an agent overhead rate for KRW-paid imports
에이전트에게 원화로 지급하는 금액에는 통관·운임이 이미 포함돼 있어
수입 부대비용률을 다시 얹으면 이중 계상이 된다.

- 설정 C29에 '에이전트 부대비용률' 추가, 기본 0%
- 매입원가의 부대비용률이 세 갈래로 갈린다
    수입 + USD/CNY : C17
    수입 + KRW     : C29  ← 신설
    국내           : C23
- 범례 블록을 두 줄 내려 자리를 만들었다 (참조되는 곳이 없어 안전)
- 상품판매가산출 안내줄에 세 비율을 모두 노출

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PfdKumnbn9qUZ8YeCg3V1y
</commit_message>
<xml_diff>
--- a/수도명가 보급형 황동수전 판매단가.xlsx
+++ b/수도명가 보급형 황동수전 판매단가.xlsx
@@ -32,7 +32,7 @@
     <numFmt numFmtId="167" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="168" formatCode="#,##0;(#,##0);-"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="35">
     <font>
       <name val="맑은 고딕"/>
       <family val="2"/>
@@ -265,6 +265,12 @@
       <color rgb="00008000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="0014606B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -798,7 +804,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="170">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1060,6 +1066,13 @@
     <xf numFmtId="167" fontId="6" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="4" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1628,6 +1641,16 @@
 절상 단위도 기준유통가와 같은 값(C27)을 씁니다.</t>
       </text>
     </comment>
+    <comment ref="C29" authorId="0" shapeId="0">
+      <text>
+        <t>부대비용률은 세 가지로 갈립니다.
+  수입 + USD/CNY : C17 (수입 부대비용률)
+  수입 + KRW     : C29 (에이전트 부대비용률) ← 이 칸
+  국내           : C23 (국내 부대비용률)
+에이전트가 통관·운임까지 포함해 원화로 청구하면 여기서 다시
+얹을 것이 없으므로 0%가 맞습니다.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -2979,8 +3002,8 @@
       <c r="C2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="B3" s="5">
-        <f>"매입원가 → 판관비 "&amp;TEXT(설정!$C$24,"0.0%")&amp;" → BEP 가격 → 영업이익 "&amp;TEXT(설정!$C$25,"0.0%")&amp;" → 기준 유통가 → (영업) 최종 유통가   ·   "&amp;설정!$C$26&amp;" 방식"</f>
+      <c r="B3" s="162">
+        <f>"매입원가 → 판관비 "&amp;TEXT(설정!$C$24,"0.0%")&amp;" → BEP 가격 → 영업이익 "&amp;TEXT(설정!$C$25,"0.0%")&amp;" → 기준 유통가 → (영업) 최종 유통가   ·   "&amp;설정!$C$26&amp;" 방식"&amp;"   ·   부대비용 수입 "&amp;TEXT(설정!$C$17,"0.0%")&amp;" / 에이전트 "&amp;TEXT(설정!$C$29,"0.0%")&amp;" / 국내 "&amp;TEXT(설정!$C$23,"0.0%")</f>
         <v/>
       </c>
       <c r="C3" s="5" t="n"/>
@@ -3134,7 +3157,7 @@
         <v>300</v>
       </c>
       <c r="I6" s="113">
-        <f>IF($D6="","",IF(OR($E6="USD",$E6="CNY"),IF(N($F6)=0,"",$F6*IF($E6="USD",설정!$C$11,설정!$C$12)*(1+IF($D6="수입",설정!$C$17,설정!$C$23))),IF(N($G6)=0,"",$G6*(1+IF($D6="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D6="","",IF(OR($E6="USD",$E6="CNY"),IF(N($F6)=0,"",$F6*IF($E6="USD",설정!$C$11,설정!$C$12)*(1+IF($D6="수입",설정!$C$17,설정!$C$23))),IF(N($G6)=0,"",$G6*(1+IF($D6="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J6" s="130" t="n"/>
@@ -3209,7 +3232,7 @@
         <v>300</v>
       </c>
       <c r="I7" s="119">
-        <f>IF($D7="","",IF(OR($E7="USD",$E7="CNY"),IF(N($F7)=0,"",$F7*IF($E7="USD",설정!$C$11,설정!$C$12)*(1+IF($D7="수입",설정!$C$17,설정!$C$23))),IF(N($G7)=0,"",$G7*(1+IF($D7="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D7="","",IF(OR($E7="USD",$E7="CNY"),IF(N($F7)=0,"",$F7*IF($E7="USD",설정!$C$11,설정!$C$12)*(1+IF($D7="수입",설정!$C$17,설정!$C$23))),IF(N($G7)=0,"",$G7*(1+IF($D7="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J7" s="135" t="n"/>
@@ -3284,7 +3307,7 @@
         <v>300</v>
       </c>
       <c r="I8" s="119">
-        <f>IF($D8="","",IF(OR($E8="USD",$E8="CNY"),IF(N($F8)=0,"",$F8*IF($E8="USD",설정!$C$11,설정!$C$12)*(1+IF($D8="수입",설정!$C$17,설정!$C$23))),IF(N($G8)=0,"",$G8*(1+IF($D8="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D8="","",IF(OR($E8="USD",$E8="CNY"),IF(N($F8)=0,"",$F8*IF($E8="USD",설정!$C$11,설정!$C$12)*(1+IF($D8="수입",설정!$C$17,설정!$C$23))),IF(N($G8)=0,"",$G8*(1+IF($D8="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J8" s="135" t="n"/>
@@ -3359,7 +3382,7 @@
         <v>300</v>
       </c>
       <c r="I9" s="119">
-        <f>IF($D9="","",IF(OR($E9="USD",$E9="CNY"),IF(N($F9)=0,"",$F9*IF($E9="USD",설정!$C$11,설정!$C$12)*(1+IF($D9="수입",설정!$C$17,설정!$C$23))),IF(N($G9)=0,"",$G9*(1+IF($D9="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D9="","",IF(OR($E9="USD",$E9="CNY"),IF(N($F9)=0,"",$F9*IF($E9="USD",설정!$C$11,설정!$C$12)*(1+IF($D9="수입",설정!$C$17,설정!$C$23))),IF(N($G9)=0,"",$G9*(1+IF($D9="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J9" s="135" t="n"/>
@@ -3434,7 +3457,7 @@
         <v>300</v>
       </c>
       <c r="I10" s="119">
-        <f>IF($D10="","",IF(OR($E10="USD",$E10="CNY"),IF(N($F10)=0,"",$F10*IF($E10="USD",설정!$C$11,설정!$C$12)*(1+IF($D10="수입",설정!$C$17,설정!$C$23))),IF(N($G10)=0,"",$G10*(1+IF($D10="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D10="","",IF(OR($E10="USD",$E10="CNY"),IF(N($F10)=0,"",$F10*IF($E10="USD",설정!$C$11,설정!$C$12)*(1+IF($D10="수입",설정!$C$17,설정!$C$23))),IF(N($G10)=0,"",$G10*(1+IF($D10="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J10" s="135" t="n"/>
@@ -3509,7 +3532,7 @@
         <v>300</v>
       </c>
       <c r="I11" s="119">
-        <f>IF($D11="","",IF(OR($E11="USD",$E11="CNY"),IF(N($F11)=0,"",$F11*IF($E11="USD",설정!$C$11,설정!$C$12)*(1+IF($D11="수입",설정!$C$17,설정!$C$23))),IF(N($G11)=0,"",$G11*(1+IF($D11="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D11="","",IF(OR($E11="USD",$E11="CNY"),IF(N($F11)=0,"",$F11*IF($E11="USD",설정!$C$11,설정!$C$12)*(1+IF($D11="수입",설정!$C$17,설정!$C$23))),IF(N($G11)=0,"",$G11*(1+IF($D11="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J11" s="135" t="n"/>
@@ -3584,7 +3607,7 @@
         <v>300</v>
       </c>
       <c r="I12" s="119">
-        <f>IF($D12="","",IF(OR($E12="USD",$E12="CNY"),IF(N($F12)=0,"",$F12*IF($E12="USD",설정!$C$11,설정!$C$12)*(1+IF($D12="수입",설정!$C$17,설정!$C$23))),IF(N($G12)=0,"",$G12*(1+IF($D12="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D12="","",IF(OR($E12="USD",$E12="CNY"),IF(N($F12)=0,"",$F12*IF($E12="USD",설정!$C$11,설정!$C$12)*(1+IF($D12="수입",설정!$C$17,설정!$C$23))),IF(N($G12)=0,"",$G12*(1+IF($D12="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J12" s="135" t="n"/>
@@ -3659,7 +3682,7 @@
         <v>300</v>
       </c>
       <c r="I13" s="119">
-        <f>IF($D13="","",IF(OR($E13="USD",$E13="CNY"),IF(N($F13)=0,"",$F13*IF($E13="USD",설정!$C$11,설정!$C$12)*(1+IF($D13="수입",설정!$C$17,설정!$C$23))),IF(N($G13)=0,"",$G13*(1+IF($D13="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D13="","",IF(OR($E13="USD",$E13="CNY"),IF(N($F13)=0,"",$F13*IF($E13="USD",설정!$C$11,설정!$C$12)*(1+IF($D13="수입",설정!$C$17,설정!$C$23))),IF(N($G13)=0,"",$G13*(1+IF($D13="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J13" s="135" t="n"/>
@@ -3720,7 +3743,7 @@
       <c r="G14" s="134" t="n"/>
       <c r="H14" s="50" t="n"/>
       <c r="I14" s="119">
-        <f>IF($D14="","",IF(OR($E14="USD",$E14="CNY"),IF(N($F14)=0,"",$F14*IF($E14="USD",설정!$C$11,설정!$C$12)*(1+IF($D14="수입",설정!$C$17,설정!$C$23))),IF(N($G14)=0,"",$G14*(1+IF($D14="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D14="","",IF(OR($E14="USD",$E14="CNY"),IF(N($F14)=0,"",$F14*IF($E14="USD",설정!$C$11,설정!$C$12)*(1+IF($D14="수입",설정!$C$17,설정!$C$23))),IF(N($G14)=0,"",$G14*(1+IF($D14="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J14" s="135" t="n"/>
@@ -3781,7 +3804,7 @@
       <c r="G15" s="134" t="n"/>
       <c r="H15" s="50" t="n"/>
       <c r="I15" s="119">
-        <f>IF($D15="","",IF(OR($E15="USD",$E15="CNY"),IF(N($F15)=0,"",$F15*IF($E15="USD",설정!$C$11,설정!$C$12)*(1+IF($D15="수입",설정!$C$17,설정!$C$23))),IF(N($G15)=0,"",$G15*(1+IF($D15="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D15="","",IF(OR($E15="USD",$E15="CNY"),IF(N($F15)=0,"",$F15*IF($E15="USD",설정!$C$11,설정!$C$12)*(1+IF($D15="수입",설정!$C$17,설정!$C$23))),IF(N($G15)=0,"",$G15*(1+IF($D15="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J15" s="135" t="n"/>
@@ -3842,7 +3865,7 @@
       <c r="G16" s="134" t="n"/>
       <c r="H16" s="50" t="n"/>
       <c r="I16" s="119">
-        <f>IF($D16="","",IF(OR($E16="USD",$E16="CNY"),IF(N($F16)=0,"",$F16*IF($E16="USD",설정!$C$11,설정!$C$12)*(1+IF($D16="수입",설정!$C$17,설정!$C$23))),IF(N($G16)=0,"",$G16*(1+IF($D16="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D16="","",IF(OR($E16="USD",$E16="CNY"),IF(N($F16)=0,"",$F16*IF($E16="USD",설정!$C$11,설정!$C$12)*(1+IF($D16="수입",설정!$C$17,설정!$C$23))),IF(N($G16)=0,"",$G16*(1+IF($D16="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J16" s="135" t="n"/>
@@ -3903,7 +3926,7 @@
       <c r="G17" s="134" t="n"/>
       <c r="H17" s="50" t="n"/>
       <c r="I17" s="119">
-        <f>IF($D17="","",IF(OR($E17="USD",$E17="CNY"),IF(N($F17)=0,"",$F17*IF($E17="USD",설정!$C$11,설정!$C$12)*(1+IF($D17="수입",설정!$C$17,설정!$C$23))),IF(N($G17)=0,"",$G17*(1+IF($D17="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D17="","",IF(OR($E17="USD",$E17="CNY"),IF(N($F17)=0,"",$F17*IF($E17="USD",설정!$C$11,설정!$C$12)*(1+IF($D17="수입",설정!$C$17,설정!$C$23))),IF(N($G17)=0,"",$G17*(1+IF($D17="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J17" s="135" t="n"/>
@@ -3964,7 +3987,7 @@
       <c r="G18" s="134" t="n"/>
       <c r="H18" s="50" t="n"/>
       <c r="I18" s="119">
-        <f>IF($D18="","",IF(OR($E18="USD",$E18="CNY"),IF(N($F18)=0,"",$F18*IF($E18="USD",설정!$C$11,설정!$C$12)*(1+IF($D18="수입",설정!$C$17,설정!$C$23))),IF(N($G18)=0,"",$G18*(1+IF($D18="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D18="","",IF(OR($E18="USD",$E18="CNY"),IF(N($F18)=0,"",$F18*IF($E18="USD",설정!$C$11,설정!$C$12)*(1+IF($D18="수입",설정!$C$17,설정!$C$23))),IF(N($G18)=0,"",$G18*(1+IF($D18="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J18" s="135" t="n"/>
@@ -4025,7 +4048,7 @@
       <c r="G19" s="134" t="n"/>
       <c r="H19" s="50" t="n"/>
       <c r="I19" s="119">
-        <f>IF($D19="","",IF(OR($E19="USD",$E19="CNY"),IF(N($F19)=0,"",$F19*IF($E19="USD",설정!$C$11,설정!$C$12)*(1+IF($D19="수입",설정!$C$17,설정!$C$23))),IF(N($G19)=0,"",$G19*(1+IF($D19="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D19="","",IF(OR($E19="USD",$E19="CNY"),IF(N($F19)=0,"",$F19*IF($E19="USD",설정!$C$11,설정!$C$12)*(1+IF($D19="수입",설정!$C$17,설정!$C$23))),IF(N($G19)=0,"",$G19*(1+IF($D19="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J19" s="135" t="n"/>
@@ -4086,7 +4109,7 @@
       <c r="G20" s="134" t="n"/>
       <c r="H20" s="50" t="n"/>
       <c r="I20" s="119">
-        <f>IF($D20="","",IF(OR($E20="USD",$E20="CNY"),IF(N($F20)=0,"",$F20*IF($E20="USD",설정!$C$11,설정!$C$12)*(1+IF($D20="수입",설정!$C$17,설정!$C$23))),IF(N($G20)=0,"",$G20*(1+IF($D20="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D20="","",IF(OR($E20="USD",$E20="CNY"),IF(N($F20)=0,"",$F20*IF($E20="USD",설정!$C$11,설정!$C$12)*(1+IF($D20="수입",설정!$C$17,설정!$C$23))),IF(N($G20)=0,"",$G20*(1+IF($D20="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J20" s="135" t="n"/>
@@ -4147,7 +4170,7 @@
       <c r="G21" s="134" t="n"/>
       <c r="H21" s="50" t="n"/>
       <c r="I21" s="119">
-        <f>IF($D21="","",IF(OR($E21="USD",$E21="CNY"),IF(N($F21)=0,"",$F21*IF($E21="USD",설정!$C$11,설정!$C$12)*(1+IF($D21="수입",설정!$C$17,설정!$C$23))),IF(N($G21)=0,"",$G21*(1+IF($D21="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D21="","",IF(OR($E21="USD",$E21="CNY"),IF(N($F21)=0,"",$F21*IF($E21="USD",설정!$C$11,설정!$C$12)*(1+IF($D21="수입",설정!$C$17,설정!$C$23))),IF(N($G21)=0,"",$G21*(1+IF($D21="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J21" s="135" t="n"/>
@@ -4208,7 +4231,7 @@
       <c r="G22" s="134" t="n"/>
       <c r="H22" s="50" t="n"/>
       <c r="I22" s="119">
-        <f>IF($D22="","",IF(OR($E22="USD",$E22="CNY"),IF(N($F22)=0,"",$F22*IF($E22="USD",설정!$C$11,설정!$C$12)*(1+IF($D22="수입",설정!$C$17,설정!$C$23))),IF(N($G22)=0,"",$G22*(1+IF($D22="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D22="","",IF(OR($E22="USD",$E22="CNY"),IF(N($F22)=0,"",$F22*IF($E22="USD",설정!$C$11,설정!$C$12)*(1+IF($D22="수입",설정!$C$17,설정!$C$23))),IF(N($G22)=0,"",$G22*(1+IF($D22="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J22" s="135" t="n"/>
@@ -4269,7 +4292,7 @@
       <c r="G23" s="134" t="n"/>
       <c r="H23" s="50" t="n"/>
       <c r="I23" s="119">
-        <f>IF($D23="","",IF(OR($E23="USD",$E23="CNY"),IF(N($F23)=0,"",$F23*IF($E23="USD",설정!$C$11,설정!$C$12)*(1+IF($D23="수입",설정!$C$17,설정!$C$23))),IF(N($G23)=0,"",$G23*(1+IF($D23="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D23="","",IF(OR($E23="USD",$E23="CNY"),IF(N($F23)=0,"",$F23*IF($E23="USD",설정!$C$11,설정!$C$12)*(1+IF($D23="수입",설정!$C$17,설정!$C$23))),IF(N($G23)=0,"",$G23*(1+IF($D23="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J23" s="135" t="n"/>
@@ -4330,7 +4353,7 @@
       <c r="G24" s="134" t="n"/>
       <c r="H24" s="50" t="n"/>
       <c r="I24" s="119">
-        <f>IF($D24="","",IF(OR($E24="USD",$E24="CNY"),IF(N($F24)=0,"",$F24*IF($E24="USD",설정!$C$11,설정!$C$12)*(1+IF($D24="수입",설정!$C$17,설정!$C$23))),IF(N($G24)=0,"",$G24*(1+IF($D24="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D24="","",IF(OR($E24="USD",$E24="CNY"),IF(N($F24)=0,"",$F24*IF($E24="USD",설정!$C$11,설정!$C$12)*(1+IF($D24="수입",설정!$C$17,설정!$C$23))),IF(N($G24)=0,"",$G24*(1+IF($D24="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J24" s="135" t="n"/>
@@ -4391,7 +4414,7 @@
       <c r="G25" s="134" t="n"/>
       <c r="H25" s="50" t="n"/>
       <c r="I25" s="119">
-        <f>IF($D25="","",IF(OR($E25="USD",$E25="CNY"),IF(N($F25)=0,"",$F25*IF($E25="USD",설정!$C$11,설정!$C$12)*(1+IF($D25="수입",설정!$C$17,설정!$C$23))),IF(N($G25)=0,"",$G25*(1+IF($D25="수입",설정!$C$17,설정!$C$23)))))</f>
+        <f>IF($D25="","",IF(OR($E25="USD",$E25="CNY"),IF(N($F25)=0,"",$F25*IF($E25="USD",설정!$C$11,설정!$C$12)*(1+IF($D25="수입",설정!$C$17,설정!$C$23))),IF(N($G25)=0,"",$G25*(1+IF($D25="수입",설정!$C$29,설정!$C$23)))))</f>
         <v/>
       </c>
       <c r="J25" s="135" t="n"/>
@@ -4495,7 +4518,7 @@
     <row r="29">
       <c r="B29" s="138" t="inlineStr">
         <is>
-          <t>② 부대비용률은 구분이 정합니다 — 수입이면 설정 C17, 국내면 설정 C23. 에이전트를 통해 원화로 결제한 수입건은 구분 '수입' + 통화 'KRW'.</t>
+          <t>② 부대비용률은 세 갈래입니다 — 수입+외화는 설정 C17, 수입+KRW(에이전트)는 설정 C29, 국내는 설정 C23.</t>
         </is>
       </c>
       <c r="C29" s="4" t="n"/>
@@ -6307,7 +6330,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D33"/>
+  <dimension ref="B2:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="3.69921875" customWidth="1" min="1" max="1"/>
@@ -6653,65 +6676,83 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="38" t="inlineStr">
+      <c r="B29" s="163" t="inlineStr">
+        <is>
+          <t>에이전트 부대비용률</t>
+        </is>
+      </c>
+      <c r="C29" s="157" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="164" t="inlineStr">
+        <is>
+          <t>구분 '수입' + 통화 'KRW' 인 건에 적용됩니다. 에이전트 지급액에 통관·운임이 포함돼 있으면 0%로 두세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="25" t="n"/>
+      <c r="D30" s="15" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="165" t="inlineStr">
         <is>
           <t>■ 범례</t>
         </is>
       </c>
-      <c r="C29" s="17" t="n"/>
-      <c r="D29" s="16" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="18" t="inlineStr">
+      <c r="C31" s="138" t="n"/>
+      <c r="D31" s="15" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="166" t="inlineStr">
         <is>
           <t>노란 채우기</t>
         </is>
       </c>
-      <c r="C30" s="25" t="inlineStr">
+      <c r="C32" s="138" t="inlineStr">
         <is>
           <t>반드시 확인하고 채워야 하는 칸</t>
         </is>
       </c>
-      <c r="D30" s="15" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="13" t="inlineStr">
+      <c r="D32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" thickBot="1">
+      <c r="B33" s="167" t="inlineStr">
         <is>
           <t>파란 글씨</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
+      <c r="C33" s="168" t="inlineStr">
         <is>
           <t>직접 입력하는 칸</t>
         </is>
       </c>
-      <c r="D31" s="15" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="13" t="inlineStr">
+      <c r="D33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="169" t="inlineStr">
         <is>
           <t>검정 글씨</t>
         </is>
       </c>
-      <c r="C32" s="96" t="inlineStr">
+      <c r="C34" s="138" t="inlineStr">
         <is>
           <t>수식 — 손대지 마세요</t>
         </is>
       </c>
-      <c r="D32" s="15" t="n"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" thickBot="1">
-      <c r="B33" s="43" t="inlineStr">
+    </row>
+    <row r="35">
+      <c r="B35" s="162" t="inlineStr">
         <is>
           <t>초록 글씨</t>
         </is>
       </c>
-      <c r="C33" s="98" t="inlineStr">
+      <c r="C35" s="138" t="inlineStr">
         <is>
           <t>다른 시트를 참조하는 수식</t>
         </is>
       </c>
-      <c r="D33" s="19" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>